<commit_message>
walk through fgsea and fry set contrasts once for every grouping
</commit_message>
<xml_diff>
--- a/03_Group_comparisons/HRvLR/03_Set_Contrasts/c_data/set_contrasts.xlsx
+++ b/03_Group_comparisons/HRvLR/03_Set_Contrasts/c_data/set_contrasts.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9834" uniqueCount="2931">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9867" uniqueCount="2951">
   <si>
     <t>sheet</t>
   </si>
@@ -8357,7 +8357,7 @@
     <t>fit</t>
   </si>
   <si>
-    <t>02_HRvLR_groups/02_Protein_Contrasts/c_data/fit.rds</t>
+    <t>03_Group_comparisons/HRvLR/02_Protein_Contrasts/c_data/fit.rds</t>
   </si>
   <si>
     <t>76d83b782ba641782d378b9ae9391e38</t>
@@ -8366,10 +8366,10 @@
     <t>design</t>
   </si>
   <si>
-    <t>02_HRvLR_groups/01_Design_Contrasts/c_data/design.rds</t>
-  </si>
-  <si>
-    <t>96d863835b9c36a26e09b4706fc4e5e6</t>
+    <t>03_Group_comparisons/HRvLR/01_Design_Contrasts/c_data/design.rds</t>
+  </si>
+  <si>
+    <t>2eec838bcc442e8a2ff1534078b14a38</t>
   </si>
   <si>
     <t>01_Processing/03_Quantification/c_data/DAList_limpa.rds</t>
@@ -8390,7 +8390,7 @@
     <t>phenotype</t>
   </si>
   <si>
-    <t>00_Input/phenotype.csv</t>
+    <t>00_Setup/Input/phenotype.csv</t>
   </si>
   <si>
     <t>5a1989db406daa0b70189a9f0df52cf3</t>
@@ -8519,12 +8519,21 @@
     <t>Github (Dustyn-T-Lewis/enrichVolcano@d3fed631f4ae95e01bd61137699313f8de5cc86e)</t>
   </si>
   <si>
+    <t>evaluate</t>
+  </si>
+  <si>
+    <t>1.0.5</t>
+  </si>
+  <si>
     <t>farver</t>
   </si>
   <si>
     <t>2.1.2</t>
   </si>
   <si>
+    <t>fastmap</t>
+  </si>
+  <si>
     <t>fastmatch</t>
   </si>
   <si>
@@ -8585,6 +8594,18 @@
     <t>1.1.4</t>
   </si>
   <si>
+    <t>htmltools</t>
+  </si>
+  <si>
+    <t>0.5.9</t>
+  </si>
+  <si>
+    <t>htmlwidgets</t>
+  </si>
+  <si>
+    <t>1.6.4</t>
+  </si>
+  <si>
     <t>IRanges</t>
   </si>
   <si>
@@ -8597,6 +8618,18 @@
     <t>1.0.14</t>
   </si>
   <si>
+    <t>jsonlite</t>
+  </si>
+  <si>
+    <t>2.0.0</t>
+  </si>
+  <si>
+    <t>knitr</t>
+  </si>
+  <si>
+    <t>1.51</t>
+  </si>
+  <si>
     <t>labeling</t>
   </si>
   <si>
@@ -8612,9 +8645,6 @@
     <t>lifecycle</t>
   </si>
   <si>
-    <t>1.0.5</t>
-  </si>
-  <si>
     <t>limma</t>
   </si>
   <si>
@@ -8639,6 +8669,12 @@
     <t>1.5.0</t>
   </si>
   <si>
+    <t>otel</t>
+  </si>
+  <si>
+    <t>0.2.0</t>
+  </si>
+  <si>
     <t>pillar</t>
   </si>
   <si>
@@ -8723,6 +8759,12 @@
     <t>CRAN (R 4.6.1)</t>
   </si>
   <si>
+    <t>rmarkdown</t>
+  </si>
+  <si>
+    <t>2.31</t>
+  </si>
+  <si>
     <t>rprojroot</t>
   </si>
   <si>
@@ -8798,6 +8840,12 @@
     <t>0.5.0</t>
   </si>
   <si>
+    <t>utf8</t>
+  </si>
+  <si>
+    <t>1.2.6</t>
+  </si>
+  <si>
     <t>vctrs</t>
   </si>
   <si>
@@ -8814,6 +8862,18 @@
   </si>
   <si>
     <t>3.0.2</t>
+  </si>
+  <si>
+    <t>xfun</t>
+  </si>
+  <si>
+    <t>0.57</t>
+  </si>
+  <si>
+    <t>yaml</t>
+  </si>
+  <si>
+    <t>2.3.12</t>
   </si>
 </sst>
 </file>
@@ -65598,7 +65658,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C71"/>
+  <dimension ref="A1:C82"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -65845,13 +65905,13 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>91</v>
+        <v>2836</v>
       </c>
       <c r="B23" t="s">
-        <v>2836</v>
+        <v>2818</v>
       </c>
       <c r="C23" t="s">
-        <v>2793</v>
+        <v>2796</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -65867,21 +65927,21 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
+        <v>91</v>
+      </c>
+      <c r="B25" t="s">
         <v>2839</v>
       </c>
-      <c r="B25" t="s">
-        <v>2840</v>
-      </c>
       <c r="C25" t="s">
-        <v>2796</v>
+        <v>2793</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
+        <v>2840</v>
+      </c>
+      <c r="B26" t="s">
         <v>2841</v>
-      </c>
-      <c r="B26" t="s">
-        <v>2842</v>
       </c>
       <c r="C26" t="s">
         <v>2796</v>
@@ -65889,10 +65949,10 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
+        <v>2842</v>
+      </c>
+      <c r="B27" t="s">
         <v>2843</v>
-      </c>
-      <c r="B27" t="s">
-        <v>2844</v>
       </c>
       <c r="C27" t="s">
         <v>2796</v>
@@ -65900,10 +65960,10 @@
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
+        <v>2844</v>
+      </c>
+      <c r="B28" t="s">
         <v>2845</v>
-      </c>
-      <c r="B28" t="s">
-        <v>2840</v>
       </c>
       <c r="C28" t="s">
         <v>2796</v>
@@ -65925,7 +65985,7 @@
         <v>2848</v>
       </c>
       <c r="B30" t="s">
-        <v>2849</v>
+        <v>2843</v>
       </c>
       <c r="C30" t="s">
         <v>2796</v>
@@ -65933,10 +65993,10 @@
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
+        <v>2849</v>
+      </c>
+      <c r="B31" t="s">
         <v>2850</v>
-      </c>
-      <c r="B31" t="s">
-        <v>2851</v>
       </c>
       <c r="C31" t="s">
         <v>2796</v>
@@ -65944,10 +66004,10 @@
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
+        <v>2851</v>
+      </c>
+      <c r="B32" t="s">
         <v>2852</v>
-      </c>
-      <c r="B32" t="s">
-        <v>2853</v>
       </c>
       <c r="C32" t="s">
         <v>2796</v>
@@ -65955,21 +66015,21 @@
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
+        <v>2853</v>
+      </c>
+      <c r="B33" t="s">
         <v>2854</v>
       </c>
-      <c r="B33" t="s">
-        <v>2855</v>
-      </c>
       <c r="C33" t="s">
-        <v>2793</v>
+        <v>2796</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
+        <v>2855</v>
+      </c>
+      <c r="B34" t="s">
         <v>2856</v>
-      </c>
-      <c r="B34" t="s">
-        <v>2857</v>
       </c>
       <c r="C34" t="s">
         <v>2796</v>
@@ -65977,10 +66037,10 @@
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
+        <v>2857</v>
+      </c>
+      <c r="B35" t="s">
         <v>2858</v>
-      </c>
-      <c r="B35" t="s">
-        <v>2859</v>
       </c>
       <c r="C35" t="s">
         <v>2796</v>
@@ -65988,10 +66048,10 @@
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
+        <v>2859</v>
+      </c>
+      <c r="B36" t="s">
         <v>2860</v>
-      </c>
-      <c r="B36" t="s">
-        <v>2861</v>
       </c>
       <c r="C36" t="s">
         <v>2796</v>
@@ -65999,32 +66059,32 @@
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
+        <v>2861</v>
+      </c>
+      <c r="B37" t="s">
         <v>2862</v>
       </c>
-      <c r="B37" t="s">
-        <v>2863</v>
-      </c>
       <c r="C37" t="s">
-        <v>2796</v>
+        <v>2793</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
+        <v>2863</v>
+      </c>
+      <c r="B38" t="s">
         <v>2864</v>
       </c>
-      <c r="B38" t="s">
-        <v>2865</v>
-      </c>
       <c r="C38" t="s">
-        <v>2793</v>
+        <v>2796</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
+        <v>2865</v>
+      </c>
+      <c r="B39" t="s">
         <v>2866</v>
-      </c>
-      <c r="B39" t="s">
-        <v>2867</v>
       </c>
       <c r="C39" t="s">
         <v>2796</v>
@@ -66032,10 +66092,10 @@
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
+        <v>2867</v>
+      </c>
+      <c r="B40" t="s">
         <v>2868</v>
-      </c>
-      <c r="B40" t="s">
-        <v>2869</v>
       </c>
       <c r="C40" t="s">
         <v>2796</v>
@@ -66043,10 +66103,10 @@
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
+        <v>2869</v>
+      </c>
+      <c r="B41" t="s">
         <v>2870</v>
-      </c>
-      <c r="B41" t="s">
-        <v>2871</v>
       </c>
       <c r="C41" t="s">
         <v>2796</v>
@@ -66054,10 +66114,10 @@
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
+        <v>2871</v>
+      </c>
+      <c r="B42" t="s">
         <v>2872</v>
-      </c>
-      <c r="B42" t="s">
-        <v>2873</v>
       </c>
       <c r="C42" t="s">
         <v>2796</v>
@@ -66065,10 +66125,10 @@
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>2874</v>
+        <v>2873</v>
       </c>
       <c r="B43" t="s">
-        <v>2875</v>
+        <v>2833</v>
       </c>
       <c r="C43" t="s">
         <v>2796</v>
@@ -66076,21 +66136,21 @@
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>2876</v>
+        <v>2874</v>
       </c>
       <c r="B44" t="s">
-        <v>2877</v>
+        <v>2875</v>
       </c>
       <c r="C44" t="s">
-        <v>2796</v>
+        <v>2793</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>2878</v>
+        <v>2876</v>
       </c>
       <c r="B45" t="s">
-        <v>2879</v>
+        <v>2877</v>
       </c>
       <c r="C45" t="s">
         <v>2796</v>
@@ -66098,10 +66158,10 @@
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>2880</v>
+        <v>2878</v>
       </c>
       <c r="B46" t="s">
-        <v>2881</v>
+        <v>2879</v>
       </c>
       <c r="C46" t="s">
         <v>2796</v>
@@ -66109,21 +66169,21 @@
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>50</v>
+        <v>2880</v>
       </c>
       <c r="B47" t="s">
-        <v>2882</v>
+        <v>2881</v>
       </c>
       <c r="C47" t="s">
-        <v>2793</v>
+        <v>2796</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
+        <v>2882</v>
+      </c>
+      <c r="B48" t="s">
         <v>2883</v>
-      </c>
-      <c r="B48" t="s">
-        <v>2884</v>
       </c>
       <c r="C48" t="s">
         <v>2796</v>
@@ -66131,10 +66191,10 @@
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
+        <v>2884</v>
+      </c>
+      <c r="B49" t="s">
         <v>2885</v>
-      </c>
-      <c r="B49" t="s">
-        <v>2886</v>
       </c>
       <c r="C49" t="s">
         <v>2796</v>
@@ -66142,10 +66202,10 @@
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
+        <v>2886</v>
+      </c>
+      <c r="B50" t="s">
         <v>2887</v>
-      </c>
-      <c r="B50" t="s">
-        <v>2888</v>
       </c>
       <c r="C50" t="s">
         <v>2796</v>
@@ -66153,10 +66213,10 @@
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
+        <v>2888</v>
+      </c>
+      <c r="B51" t="s">
         <v>2889</v>
-      </c>
-      <c r="B51" t="s">
-        <v>2890</v>
       </c>
       <c r="C51" t="s">
         <v>2796</v>
@@ -66164,10 +66224,10 @@
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
+        <v>2890</v>
+      </c>
+      <c r="B52" t="s">
         <v>2891</v>
-      </c>
-      <c r="B52" t="s">
-        <v>2892</v>
       </c>
       <c r="C52" t="s">
         <v>2796</v>
@@ -66175,10 +66235,10 @@
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
+        <v>2892</v>
+      </c>
+      <c r="B53" t="s">
         <v>2893</v>
-      </c>
-      <c r="B53" t="s">
-        <v>2894</v>
       </c>
       <c r="C53" t="s">
         <v>2796</v>
@@ -66186,32 +66246,32 @@
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>2895</v>
+        <v>50</v>
       </c>
       <c r="B54" t="s">
-        <v>2896</v>
+        <v>2894</v>
       </c>
       <c r="C54" t="s">
-        <v>2796</v>
+        <v>2793</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>2897</v>
+        <v>2895</v>
       </c>
       <c r="B55" t="s">
-        <v>2898</v>
+        <v>2896</v>
       </c>
       <c r="C55" t="s">
-        <v>2899</v>
+        <v>2796</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>2900</v>
+        <v>2897</v>
       </c>
       <c r="B56" t="s">
-        <v>2901</v>
+        <v>2898</v>
       </c>
       <c r="C56" t="s">
         <v>2796</v>
@@ -66219,21 +66279,21 @@
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>2902</v>
+        <v>2899</v>
       </c>
       <c r="B57" t="s">
-        <v>2903</v>
+        <v>2900</v>
       </c>
       <c r="C57" t="s">
-        <v>2793</v>
+        <v>2796</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>2904</v>
+        <v>2901</v>
       </c>
       <c r="B58" t="s">
-        <v>2905</v>
+        <v>2902</v>
       </c>
       <c r="C58" t="s">
         <v>2796</v>
@@ -66241,10 +66301,10 @@
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>2906</v>
+        <v>2903</v>
       </c>
       <c r="B59" t="s">
-        <v>2907</v>
+        <v>2904</v>
       </c>
       <c r="C59" t="s">
         <v>2796</v>
@@ -66252,10 +66312,10 @@
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>2908</v>
+        <v>2905</v>
       </c>
       <c r="B60" t="s">
-        <v>2909</v>
+        <v>2906</v>
       </c>
       <c r="C60" t="s">
         <v>2796</v>
@@ -66263,10 +66323,10 @@
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>2910</v>
+        <v>2907</v>
       </c>
       <c r="B61" t="s">
-        <v>2911</v>
+        <v>2908</v>
       </c>
       <c r="C61" t="s">
         <v>2796</v>
@@ -66274,21 +66334,21 @@
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>2912</v>
+        <v>2909</v>
       </c>
       <c r="B62" t="s">
-        <v>2913</v>
+        <v>2910</v>
       </c>
       <c r="C62" t="s">
-        <v>2796</v>
+        <v>2911</v>
       </c>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>2914</v>
+        <v>2912</v>
       </c>
       <c r="B63" t="s">
-        <v>2915</v>
+        <v>2913</v>
       </c>
       <c r="C63" t="s">
         <v>2796</v>
@@ -66296,10 +66356,10 @@
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>2916</v>
+        <v>2914</v>
       </c>
       <c r="B64" t="s">
-        <v>2917</v>
+        <v>2915</v>
       </c>
       <c r="C64" t="s">
         <v>2796</v>
@@ -66307,21 +66367,21 @@
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>2918</v>
+        <v>2916</v>
       </c>
       <c r="B65" t="s">
-        <v>2919</v>
+        <v>2917</v>
       </c>
       <c r="C65" t="s">
-        <v>2796</v>
+        <v>2793</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>2920</v>
+        <v>2918</v>
       </c>
       <c r="B66" t="s">
-        <v>2921</v>
+        <v>2919</v>
       </c>
       <c r="C66" t="s">
         <v>2796</v>
@@ -66329,10 +66389,10 @@
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>2922</v>
+        <v>2920</v>
       </c>
       <c r="B67" t="s">
-        <v>2828</v>
+        <v>2921</v>
       </c>
       <c r="C67" t="s">
         <v>2796</v>
@@ -66340,10 +66400,10 @@
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
+        <v>2922</v>
+      </c>
+      <c r="B68" t="s">
         <v>2923</v>
-      </c>
-      <c r="B68" t="s">
-        <v>2924</v>
       </c>
       <c r="C68" t="s">
         <v>2796</v>
@@ -66351,10 +66411,10 @@
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
+        <v>2924</v>
+      </c>
+      <c r="B69" t="s">
         <v>2925</v>
-      </c>
-      <c r="B69" t="s">
-        <v>2926</v>
       </c>
       <c r="C69" t="s">
         <v>2796</v>
@@ -66362,10 +66422,10 @@
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
+        <v>2926</v>
+      </c>
+      <c r="B70" t="s">
         <v>2927</v>
-      </c>
-      <c r="B70" t="s">
-        <v>2928</v>
       </c>
       <c r="C70" t="s">
         <v>2796</v>
@@ -66373,12 +66433,133 @@
     </row>
     <row r="71" spans="1:3">
       <c r="A71" t="s">
+        <v>2928</v>
+      </c>
+      <c r="B71" t="s">
         <v>2929</v>
       </c>
-      <c r="B71" t="s">
+      <c r="C71" t="s">
+        <v>2796</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3">
+      <c r="A72" t="s">
         <v>2930</v>
       </c>
-      <c r="C71" t="s">
+      <c r="B72" t="s">
+        <v>2931</v>
+      </c>
+      <c r="C72" t="s">
+        <v>2796</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3">
+      <c r="A73" t="s">
+        <v>2932</v>
+      </c>
+      <c r="B73" t="s">
+        <v>2933</v>
+      </c>
+      <c r="C73" t="s">
+        <v>2796</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3">
+      <c r="A74" t="s">
+        <v>2934</v>
+      </c>
+      <c r="B74" t="s">
+        <v>2935</v>
+      </c>
+      <c r="C74" t="s">
+        <v>2796</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3">
+      <c r="A75" t="s">
+        <v>2936</v>
+      </c>
+      <c r="B75" t="s">
+        <v>2828</v>
+      </c>
+      <c r="C75" t="s">
+        <v>2796</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3">
+      <c r="A76" t="s">
+        <v>2937</v>
+      </c>
+      <c r="B76" t="s">
+        <v>2938</v>
+      </c>
+      <c r="C76" t="s">
+        <v>2796</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3">
+      <c r="A77" t="s">
+        <v>2939</v>
+      </c>
+      <c r="B77" t="s">
+        <v>2940</v>
+      </c>
+      <c r="C77" t="s">
+        <v>2796</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3">
+      <c r="A78" t="s">
+        <v>2941</v>
+      </c>
+      <c r="B78" t="s">
+        <v>2942</v>
+      </c>
+      <c r="C78" t="s">
+        <v>2796</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3">
+      <c r="A79" t="s">
+        <v>2943</v>
+      </c>
+      <c r="B79" t="s">
+        <v>2944</v>
+      </c>
+      <c r="C79" t="s">
+        <v>2796</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3">
+      <c r="A80" t="s">
+        <v>2945</v>
+      </c>
+      <c r="B80" t="s">
+        <v>2946</v>
+      </c>
+      <c r="C80" t="s">
+        <v>2796</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3">
+      <c r="A81" t="s">
+        <v>2947</v>
+      </c>
+      <c r="B81" t="s">
+        <v>2948</v>
+      </c>
+      <c r="C81" t="s">
+        <v>2796</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3">
+      <c r="A82" t="s">
+        <v>2949</v>
+      </c>
+      <c r="B82" t="s">
+        <v>2950</v>
+      </c>
+      <c r="C82" t="s">
         <v>2796</v>
       </c>
     </row>

</xml_diff>